<commit_message>
few formatting related changes and reference links for further reading in readmes and refined the readmes, and removed too much hints/pseudocodes from the starter. this is the large commit with lots of these minor changes.
</commit_message>
<xml_diff>
--- a/02_ai-risk-framework-implementation-nist-ai-rmf/exercises/starter/risk_assessment.xlsx
+++ b/02_ai-risk-framework-implementation-nist-ai-rmf/exercises/starter/risk_assessment.xlsx
@@ -1008,12 +1008,12 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H5" s="12">
@@ -1026,22 +1026,22 @@
       </c>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H6" s="12">
@@ -1091,22 +1091,22 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M6" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1138,12 +1138,12 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H7" s="12">
@@ -1156,22 +1156,22 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1203,12 +1203,12 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H8" s="12">
@@ -1221,22 +1221,22 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M8" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H9" s="12">
@@ -1286,22 +1286,22 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H10" s="12">
@@ -1351,22 +1351,22 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M10" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1398,12 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H11" s="12">
@@ -1416,22 +1416,22 @@
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1484,22 +1484,22 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M12" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H13" s="12">
@@ -1549,22 +1549,22 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M13" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1596,12 +1596,12 @@
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H14" s="12">
@@ -1614,22 +1614,22 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M14" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1682,22 +1682,22 @@
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
         </is>
       </c>
       <c r="H16" s="12">
@@ -1747,43 +1747,217 @@
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
         </is>
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
         </is>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
         </is>
       </c>
       <c r="M16" s="12" t="inlineStr">
         <is>
-          <t>[Your response here]</t>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>R016</t>
         </is>
       </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>GENAI-SPECIFIC: Hallucinated fraud explanations - System generates plausible but fabricated reasoning when flagging transactions, misleading analysts</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Data Science Lead</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
+        </is>
+      </c>
+      <c r="H17" s="12">
+        <f>IF(F17="","",F17*G17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="12">
+        <f>IF(F17="","",IF(H17&gt;=15,"Critical",IF(H17&gt;=10,"High",IF(H17&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>R017</t>
         </is>
       </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>GENAI-SPECIFIC: Prompt injection vulnerabilities - Adversarial prompts manipulate fraud detection outputs, causing false positives or false negatives</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>ML Security Engineer</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
+        </is>
+      </c>
+      <c r="H18" s="12">
+        <f>IF(F18="","",F18*G18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="12">
+        <f>IF(F18="","",IF(H18&gt;=15,"Critical",IF(H18&gt;=10,"High",IF(H18&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
+        </is>
+      </c>
+      <c r="M18" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>R018</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Govern</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>GENAI-SPECIFIC: Training data poisoning - Contaminated training data causes systematic misclassifications in fraud detection model</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Data Science Lead</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 reflecting how severe this risk's worst-case outcome would be for FinGuard (financial loss, customer harm, regulatory penalty); see the Scoring Rubric sheet for what each level means.]</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — score 1-5 estimating how likely this risk is to materialize within ~12 months given the scenario context; see the Scoring Rubric sheet for level definitions.]</t>
+        </is>
+      </c>
+      <c r="H19" s="12">
+        <f>IF(F19="","",F19*G19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="12">
+        <f>IF(F19="","",IF(H19&gt;=15,"Critical",IF(H19&gt;=10,"High",IF(H19&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — name 2-3 specific controls that would reduce this risk's likelihood or impact (think monitoring, validation, governance, human-in-the-loop, redundancy); match them to the risk type.]</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>[Your response here — assign Critical / High / Medium / Low based on the Risk Score band and business urgency; cross-check against the Scoring Rubric thresholds.]</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — pick the current state of this mitigation: Open, In Progress, or Closed (most starter risks will be Open).]</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr">
+        <is>
+          <t>[Your response here — propose a realistic target completion date (e.g., "Q2 2026") or "TBD" if owner needs to scope first; align urgency with the Priority you assigned.]</t>
         </is>
       </c>
     </row>
@@ -1987,7 +2161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2015,7 +2189,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Risk Register'!A2:A16)</f>
+        <f>COUNTA('Risk Register'!A2:A19)</f>
         <v/>
       </c>
     </row>
@@ -2026,7 +2200,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Risk Register'!I2:I16,"Critical")</f>
+        <f>COUNTIF('Risk Register'!I2:I19,"Critical")</f>
         <v/>
       </c>
     </row>
@@ -2037,7 +2211,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Risk Register'!I2:I16,"High")</f>
+        <f>COUNTIF('Risk Register'!I2:I19,"High")</f>
         <v/>
       </c>
     </row>
@@ -2048,7 +2222,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Risk Register'!I2:I16,"Medium")</f>
+        <f>COUNTIF('Risk Register'!I2:I19,"Medium")</f>
         <v/>
       </c>
     </row>
@@ -2059,7 +2233,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF('Risk Register'!I2:I16,"Low")</f>
+        <f>COUNTIF('Risk Register'!I2:I19,"Low")</f>
         <v/>
       </c>
     </row>
@@ -2077,7 +2251,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Risk Register'!C2:C16,"Technical")</f>
+        <f>COUNTIF('Risk Register'!C2:C19,"Technical")</f>
         <v/>
       </c>
     </row>
@@ -2088,7 +2262,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Risk Register'!C2:C16,"Ethical")</f>
+        <f>COUNTIF('Risk Register'!C2:C19,"Ethical")</f>
         <v/>
       </c>
     </row>
@@ -2099,7 +2273,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Risk Register'!C2:C16,"Legal")</f>
+        <f>COUNTIF('Risk Register'!C2:C19,"Legal")</f>
         <v/>
       </c>
     </row>
@@ -2110,7 +2284,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF('Risk Register'!C2:C16,"Operational")</f>
+        <f>COUNTIF('Risk Register'!C2:C19,"Operational")</f>
         <v/>
       </c>
     </row>
@@ -2128,7 +2302,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF('Risk Register'!B2:B16,"Govern")</f>
+        <f>COUNTIF('Risk Register'!B2:B19,"Govern")</f>
         <v/>
       </c>
     </row>
@@ -2139,7 +2313,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Risk Register'!B2:B16,"Map")</f>
+        <f>COUNTIF('Risk Register'!B2:B19,"Map")</f>
         <v/>
       </c>
     </row>
@@ -2150,7 +2324,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Risk Register'!B2:B16,"Measure")</f>
+        <f>COUNTIF('Risk Register'!B2:B19,"Measure")</f>
         <v/>
       </c>
     </row>
@@ -2161,28 +2335,77 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF('Risk Register'!B2:B16,"Manage")</f>
+        <f>COUNTIF('Risk Register'!B2:B19,"Manage")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>KEY FINDINGS</t>
+          <t>TOP 5 PRIORITY RISKS</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Hint: Summarize the overall risk posture — what is the biggest concern?</t>
+          <t>1. [Your response here — Risk #1: list Risk ID, short name, Risk Level, and Impact x Likelihood for the highest-scored risk in your register.]</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Hint: What patterns do you see across categories? Any clusters of risk?</t>
+          <t>2. [Your response here — Risk #2: same format as above, next-highest scored risk; break ties by business impact.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3. [Your response here — Risk #3: same format; consider both Critical risks and any High risks with strategic significance.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4. [Your response here — Risk #4: same format; remember GenAI-specific and legal risks may rank here.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5. [Your response here — Risk #5: same format; round out the top 5 with the next priority risk an executive should track.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>KEY FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[Your response here — one sentence summarizing FinGuard's overall risk posture: which risk category (technical, ethical, legal, operational) dominates and why it matters to leadership?]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[Your response here — call out patterns or clusters across NIST AI RMF functions or risk categories (e.g., concentration in Measure, multiple bias-related risks); reference the counts in B5:B20.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[Your response here — one sentence on legal/regulatory exposure for executives, naming the specific regimes at play (e.g., GDPR Article 22, EU AI Act high-risk obligations).]</t>
         </is>
       </c>
     </row>

</xml_diff>